<commit_message>
2/09: WM San Cristobal bloqueada (fantasma 124 u) → pedido 161 cajas Q66,269 (Excel/PDF/CSV/bodega regenerados) · sala: causa Pinula (vale), A11 nota prioritaria, +WM SC · REPORTE-EQUIPO-GSP-SEM630 (acuerdos reunion, hallazgos, 16 sin contar, en ruta, formato vencimientos)
</commit_message>
<xml_diff>
--- a/expediente-walmart-2026/pedido-refuerzo/SUGERIDO_WALMART_2026-08-31.xlsx
+++ b/expediente-walmart-2026/pedido-refuerzo/SUGERIDO_WALMART_2026-08-31.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P129"/>
+  <dimension ref="A1:P123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3301,11 +3301,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HB SESSION LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>75437617</v>
+        <v>75437612</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -3313,13 +3313,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>16</v>
+        <v>43.8</v>
       </c>
       <c r="E48" t="n">
-        <v>2.098575</v>
+        <v>5.74485</v>
       </c>
       <c r="F48" t="n">
-        <v>400568690161</v>
+        <v>72734400408</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3339,11 +3339,11 @@
         <v>20</v>
       </c>
       <c r="L48" t="n">
-        <v>1054</v>
+        <v>4173</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>WALMART SAN CRISTóBAL</t>
+          <t>PAIZ SANTA AMELIA</t>
         </is>
       </c>
       <c r="N48" t="n">
@@ -3361,11 +3361,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NC SCRIMSHAW LATA</t>
+          <t>BELHAVEN BEST LATA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>75437612</v>
+        <v>75437618</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -3373,13 +3373,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>43.8</v>
+        <v>18.25</v>
       </c>
       <c r="E49" t="n">
-        <v>5.74485</v>
+        <v>2.393687</v>
       </c>
       <c r="F49" t="n">
-        <v>72734400408</v>
+        <v>501054930410</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3399,22 +3399,22 @@
         <v>20</v>
       </c>
       <c r="L49" t="n">
-        <v>4173</v>
+        <v>457</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>PAIZ SANTA AMELIA</t>
+          <t>PAIZ ASUNCION</t>
         </is>
       </c>
       <c r="N49" t="n">
         <v>0</v>
       </c>
       <c r="O49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>MEDICIÓN · sin existencias en RL sem 202630 · piso de 1 caja para lectura de demanda</t>
+          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
         </is>
       </c>
     </row>
@@ -3459,11 +3459,11 @@
         <v>20</v>
       </c>
       <c r="L50" t="n">
-        <v>457</v>
+        <v>491</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>PAIZ ASUNCION</t>
+          <t>PAIZ COBAN</t>
         </is>
       </c>
       <c r="N50" t="n">
@@ -3519,11 +3519,11 @@
         <v>20</v>
       </c>
       <c r="L51" t="n">
-        <v>491</v>
+        <v>4087</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>PAIZ COBAN</t>
+          <t>PAIZ EL NARANJO</t>
         </is>
       </c>
       <c r="N51" t="n">
@@ -3579,11 +3579,11 @@
         <v>20</v>
       </c>
       <c r="L52" t="n">
-        <v>4087</v>
+        <v>180</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>PAIZ EL NARANJO</t>
+          <t>PAIZ HUEHUETENANGO</t>
         </is>
       </c>
       <c r="N52" t="n">
@@ -3639,11 +3639,11 @@
         <v>20</v>
       </c>
       <c r="L53" t="n">
-        <v>180</v>
+        <v>4491</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>PAIZ HUEHUETENANGO</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N53" t="n">
@@ -3699,11 +3699,11 @@
         <v>20</v>
       </c>
       <c r="L54" t="n">
-        <v>4491</v>
+        <v>47</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>PAIZ MONTBLANC</t>
         </is>
       </c>
       <c r="N54" t="n">
@@ -3759,11 +3759,11 @@
         <v>20</v>
       </c>
       <c r="L55" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>PAIZ MONTBLANC</t>
+          <t>PAIZ PETAPA</t>
         </is>
       </c>
       <c r="N55" t="n">
@@ -3819,11 +3819,11 @@
         <v>20</v>
       </c>
       <c r="L56" t="n">
-        <v>35</v>
+        <v>458</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>PAIZ PETAPA</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N56" t="n">
@@ -3879,11 +3879,11 @@
         <v>20</v>
       </c>
       <c r="L57" t="n">
-        <v>458</v>
+        <v>169</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
+          <t>PAIZ SAN CRISTOBAL</t>
         </is>
       </c>
       <c r="N57" t="n">
@@ -3939,11 +3939,11 @@
         <v>20</v>
       </c>
       <c r="L58" t="n">
-        <v>169</v>
+        <v>34</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>PAIZ SAN CRISTOBAL</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -3999,11 +3999,11 @@
         <v>20</v>
       </c>
       <c r="L59" t="n">
-        <v>34</v>
+        <v>4414</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>PAIZ UTATLAN</t>
+          <t>WM ATANASIO TZUL</t>
         </is>
       </c>
       <c r="N59" t="n">
@@ -4059,11 +4059,11 @@
         <v>20</v>
       </c>
       <c r="L60" t="n">
-        <v>1054</v>
+        <v>4116</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>WALMART SAN CRISTóBAL</t>
+          <t>WM MIXCO</t>
         </is>
       </c>
       <c r="N60" t="n">
@@ -4119,11 +4119,11 @@
         <v>20</v>
       </c>
       <c r="L61" t="n">
-        <v>4414</v>
+        <v>4370</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>WM ATANASIO TZUL</t>
+          <t>WM PROCERES</t>
         </is>
       </c>
       <c r="N61" t="n">
@@ -4179,11 +4179,11 @@
         <v>20</v>
       </c>
       <c r="L62" t="n">
-        <v>4116</v>
+        <v>1087</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>WM MIXCO</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N62" t="n">
@@ -4239,11 +4239,11 @@
         <v>20</v>
       </c>
       <c r="L63" t="n">
-        <v>4370</v>
+        <v>460</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>WM PROCERES</t>
+          <t>WM XELA</t>
         </is>
       </c>
       <c r="N63" t="n">
@@ -4261,11 +4261,11 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BELHAVEN BEST LATA</t>
+          <t>BELHAVEN BLACK LATA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>75437618</v>
+        <v>75437619</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -4279,7 +4279,7 @@
         <v>2.393687</v>
       </c>
       <c r="F64" t="n">
-        <v>501054930410</v>
+        <v>501054930472</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -4299,11 +4299,11 @@
         <v>20</v>
       </c>
       <c r="L64" t="n">
-        <v>1087</v>
+        <v>457</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
+          <t>PAIZ ASUNCION</t>
         </is>
       </c>
       <c r="N64" t="n">
@@ -4321,11 +4321,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BELHAVEN BEST LATA</t>
+          <t>BELHAVEN BLACK LATA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>75437618</v>
+        <v>75437619</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
         <v>2.393687</v>
       </c>
       <c r="F65" t="n">
-        <v>501054930410</v>
+        <v>501054930472</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -4359,11 +4359,11 @@
         <v>20</v>
       </c>
       <c r="L65" t="n">
-        <v>460</v>
+        <v>491</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>WM XELA</t>
+          <t>PAIZ COBAN</t>
         </is>
       </c>
       <c r="N65" t="n">
@@ -4419,11 +4419,11 @@
         <v>20</v>
       </c>
       <c r="L66" t="n">
-        <v>457</v>
+        <v>727</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>PAIZ ASUNCION</t>
+          <t>PAIZ COLONIA VISTA HERMOS</t>
         </is>
       </c>
       <c r="N66" t="n">
@@ -4479,11 +4479,11 @@
         <v>20</v>
       </c>
       <c r="L67" t="n">
-        <v>491</v>
+        <v>180</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>PAIZ COBAN</t>
+          <t>PAIZ HUEHUETENANGO</t>
         </is>
       </c>
       <c r="N67" t="n">
@@ -4539,11 +4539,11 @@
         <v>20</v>
       </c>
       <c r="L68" t="n">
-        <v>727</v>
+        <v>4491</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>PAIZ COLONIA VISTA HERMOS</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N68" t="n">
@@ -4599,11 +4599,11 @@
         <v>20</v>
       </c>
       <c r="L69" t="n">
-        <v>180</v>
+        <v>47</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>PAIZ HUEHUETENANGO</t>
+          <t>PAIZ MONTBLANC</t>
         </is>
       </c>
       <c r="N69" t="n">
@@ -4659,11 +4659,11 @@
         <v>20</v>
       </c>
       <c r="L70" t="n">
-        <v>4491</v>
+        <v>20</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>PAIZ MONTUFAR</t>
         </is>
       </c>
       <c r="N70" t="n">
@@ -4719,11 +4719,11 @@
         <v>20</v>
       </c>
       <c r="L71" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>PAIZ MONTBLANC</t>
+          <t>PAIZ PETAPA</t>
         </is>
       </c>
       <c r="N71" t="n">
@@ -4779,11 +4779,11 @@
         <v>20</v>
       </c>
       <c r="L72" t="n">
-        <v>20</v>
+        <v>458</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>PAIZ MONTUFAR</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N72" t="n">
@@ -4839,11 +4839,11 @@
         <v>20</v>
       </c>
       <c r="L73" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>PAIZ PETAPA</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N73" t="n">
@@ -4899,11 +4899,11 @@
         <v>20</v>
       </c>
       <c r="L74" t="n">
-        <v>458</v>
+        <v>4414</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
+          <t>WM ATANASIO TZUL</t>
         </is>
       </c>
       <c r="N74" t="n">
@@ -4959,11 +4959,11 @@
         <v>20</v>
       </c>
       <c r="L75" t="n">
-        <v>34</v>
+        <v>4037</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>PAIZ UTATLAN</t>
+          <t>WM DEL NORTE</t>
         </is>
       </c>
       <c r="N75" t="n">
@@ -5019,11 +5019,11 @@
         <v>20</v>
       </c>
       <c r="L76" t="n">
-        <v>1054</v>
+        <v>4116</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>WALMART SAN CRISTóBAL</t>
+          <t>WM MIXCO</t>
         </is>
       </c>
       <c r="N76" t="n">
@@ -5079,11 +5079,11 @@
         <v>20</v>
       </c>
       <c r="L77" t="n">
-        <v>4414</v>
+        <v>4370</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>WM ATANASIO TZUL</t>
+          <t>WM PROCERES</t>
         </is>
       </c>
       <c r="N77" t="n">
@@ -5139,11 +5139,11 @@
         <v>20</v>
       </c>
       <c r="L78" t="n">
-        <v>4037</v>
+        <v>164</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>WM DEL NORTE</t>
+          <t>WM PUERTA PARADA</t>
         </is>
       </c>
       <c r="N78" t="n">
@@ -5199,11 +5199,11 @@
         <v>20</v>
       </c>
       <c r="L79" t="n">
-        <v>4116</v>
+        <v>1087</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>WM MIXCO</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N79" t="n">
@@ -5259,11 +5259,11 @@
         <v>20</v>
       </c>
       <c r="L80" t="n">
-        <v>4370</v>
+        <v>460</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>WM PROCERES</t>
+          <t>WM XELA</t>
         </is>
       </c>
       <c r="N80" t="n">
@@ -5281,11 +5281,11 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BELHAVEN BLACK LATA</t>
+          <t>BELHAVEN MCCALLUMS</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>75437619</v>
+        <v>75437620</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -5299,7 +5299,7 @@
         <v>2.393687</v>
       </c>
       <c r="F81" t="n">
-        <v>501054930472</v>
+        <v>501054930713</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -5319,11 +5319,11 @@
         <v>20</v>
       </c>
       <c r="L81" t="n">
-        <v>164</v>
+        <v>457</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>WM PUERTA PARADA</t>
+          <t>PAIZ ASUNCION</t>
         </is>
       </c>
       <c r="N81" t="n">
@@ -5341,11 +5341,11 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BELHAVEN BLACK LATA</t>
+          <t>BELHAVEN MCCALLUMS</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>75437619</v>
+        <v>75437620</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>2.393687</v>
       </c>
       <c r="F82" t="n">
-        <v>501054930472</v>
+        <v>501054930713</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -5379,11 +5379,11 @@
         <v>20</v>
       </c>
       <c r="L82" t="n">
-        <v>1087</v>
+        <v>4126</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
+          <t>PAIZ CHIQUIMULA PRADERA</t>
         </is>
       </c>
       <c r="N82" t="n">
@@ -5401,11 +5401,11 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BELHAVEN BLACK LATA</t>
+          <t>BELHAVEN MCCALLUMS</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>75437619</v>
+        <v>75437620</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         <v>2.393687</v>
       </c>
       <c r="F83" t="n">
-        <v>501054930472</v>
+        <v>501054930713</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -5439,11 +5439,11 @@
         <v>20</v>
       </c>
       <c r="L83" t="n">
-        <v>460</v>
+        <v>491</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>WM XELA</t>
+          <t>PAIZ COBAN</t>
         </is>
       </c>
       <c r="N83" t="n">
@@ -5499,11 +5499,11 @@
         <v>20</v>
       </c>
       <c r="L84" t="n">
-        <v>457</v>
+        <v>727</v>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>PAIZ ASUNCION</t>
+          <t>PAIZ COLONIA VISTA HERMOS</t>
         </is>
       </c>
       <c r="N84" t="n">
@@ -5559,11 +5559,11 @@
         <v>20</v>
       </c>
       <c r="L85" t="n">
-        <v>4126</v>
+        <v>180</v>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>PAIZ CHIQUIMULA PRADERA</t>
+          <t>PAIZ HUEHUETENANGO</t>
         </is>
       </c>
       <c r="N85" t="n">
@@ -5619,11 +5619,11 @@
         <v>20</v>
       </c>
       <c r="L86" t="n">
-        <v>491</v>
+        <v>4491</v>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>PAIZ COBAN</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N86" t="n">
@@ -5679,11 +5679,11 @@
         <v>20</v>
       </c>
       <c r="L87" t="n">
-        <v>727</v>
+        <v>47</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>PAIZ COLONIA VISTA HERMOS</t>
+          <t>PAIZ MONTBLANC</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -5739,11 +5739,11 @@
         <v>20</v>
       </c>
       <c r="L88" t="n">
-        <v>180</v>
+        <v>35</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>PAIZ HUEHUETENANGO</t>
+          <t>PAIZ PETAPA</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -5799,11 +5799,11 @@
         <v>20</v>
       </c>
       <c r="L89" t="n">
-        <v>4491</v>
+        <v>458</v>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N89" t="n">
@@ -5859,11 +5859,11 @@
         <v>20</v>
       </c>
       <c r="L90" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>PAIZ MONTBLANC</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N90" t="n">
@@ -5919,11 +5919,11 @@
         <v>20</v>
       </c>
       <c r="L91" t="n">
-        <v>35</v>
+        <v>4414</v>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>PAIZ PETAPA</t>
+          <t>WM ATANASIO TZUL</t>
         </is>
       </c>
       <c r="N91" t="n">
@@ -5979,11 +5979,11 @@
         <v>20</v>
       </c>
       <c r="L92" t="n">
-        <v>458</v>
+        <v>4116</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
+          <t>WM MIXCO</t>
         </is>
       </c>
       <c r="N92" t="n">
@@ -6039,11 +6039,11 @@
         <v>20</v>
       </c>
       <c r="L93" t="n">
-        <v>34</v>
+        <v>1087</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>PAIZ UTATLAN</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N93" t="n">
@@ -6099,11 +6099,11 @@
         <v>20</v>
       </c>
       <c r="L94" t="n">
-        <v>1054</v>
+        <v>460</v>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>WALMART SAN CRISTóBAL</t>
+          <t>WM XELA</t>
         </is>
       </c>
       <c r="N94" t="n">
@@ -6121,11 +6121,11 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BELHAVEN MCCALLUMS</t>
+          <t>HB HELLES LAGER LATA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>75437620</v>
+        <v>75437615</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -6133,13 +6133,13 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>18.25</v>
+        <v>16</v>
       </c>
       <c r="E95" t="n">
-        <v>2.393687</v>
+        <v>2.098575</v>
       </c>
       <c r="F95" t="n">
-        <v>501054930713</v>
+        <v>400568600172</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -6159,11 +6159,11 @@
         <v>20</v>
       </c>
       <c r="L95" t="n">
-        <v>4414</v>
+        <v>457</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>WM ATANASIO TZUL</t>
+          <t>PAIZ ASUNCION</t>
         </is>
       </c>
       <c r="N95" t="n">
@@ -6181,11 +6181,11 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BELHAVEN MCCALLUMS</t>
+          <t>HB HELLES LAGER LATA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>75437620</v>
+        <v>75437615</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -6193,13 +6193,13 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>18.25</v>
+        <v>16</v>
       </c>
       <c r="E96" t="n">
-        <v>2.393687</v>
+        <v>2.098575</v>
       </c>
       <c r="F96" t="n">
-        <v>501054930713</v>
+        <v>400568600172</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -6219,11 +6219,11 @@
         <v>20</v>
       </c>
       <c r="L96" t="n">
-        <v>4116</v>
+        <v>4491</v>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>WM MIXCO</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N96" t="n">
@@ -6241,11 +6241,11 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>BELHAVEN MCCALLUMS</t>
+          <t>HB HELLES LAGER LATA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>75437620</v>
+        <v>75437615</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -6253,13 +6253,13 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>18.25</v>
+        <v>16</v>
       </c>
       <c r="E97" t="n">
-        <v>2.393687</v>
+        <v>2.098575</v>
       </c>
       <c r="F97" t="n">
-        <v>501054930713</v>
+        <v>400568600172</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -6279,11 +6279,11 @@
         <v>20</v>
       </c>
       <c r="L97" t="n">
-        <v>1087</v>
+        <v>164</v>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
+          <t>WM PUERTA PARADA</t>
         </is>
       </c>
       <c r="N97" t="n">
@@ -6301,11 +6301,11 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BELHAVEN MCCALLUMS</t>
+          <t>HB HELLES LAGER LATA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>75437620</v>
+        <v>75437615</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -6313,13 +6313,13 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>18.25</v>
+        <v>16</v>
       </c>
       <c r="E98" t="n">
-        <v>2.393687</v>
+        <v>2.098575</v>
       </c>
       <c r="F98" t="n">
-        <v>501054930713</v>
+        <v>400568600172</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -6339,11 +6339,11 @@
         <v>20</v>
       </c>
       <c r="L98" t="n">
-        <v>460</v>
+        <v>1087</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>WM XELA</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N98" t="n">
@@ -6361,11 +6361,11 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>HB HELLES LAGER LATA</t>
+          <t>HB SESSION LATA</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>75437615</v>
+        <v>75437617</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -6379,7 +6379,7 @@
         <v>2.098575</v>
       </c>
       <c r="F99" t="n">
-        <v>400568600172</v>
+        <v>400568690161</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -6399,11 +6399,11 @@
         <v>20</v>
       </c>
       <c r="L99" t="n">
-        <v>457</v>
+        <v>4126</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>PAIZ ASUNCION</t>
+          <t>PAIZ CHIQUIMULA PRADERA</t>
         </is>
       </c>
       <c r="N99" t="n">
@@ -6421,11 +6421,11 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>HB HELLES LAGER LATA</t>
+          <t>HB SESSION LATA</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>75437615</v>
+        <v>75437617</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -6439,7 +6439,7 @@
         <v>2.098575</v>
       </c>
       <c r="F100" t="n">
-        <v>400568600172</v>
+        <v>400568690161</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -6459,11 +6459,11 @@
         <v>20</v>
       </c>
       <c r="L100" t="n">
-        <v>4491</v>
+        <v>727</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>PAIZ COLONIA VISTA HERMOS</t>
         </is>
       </c>
       <c r="N100" t="n">
@@ -6481,11 +6481,11 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HB HELLES LAGER LATA</t>
+          <t>HB SESSION LATA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>75437615</v>
+        <v>75437617</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -6499,7 +6499,7 @@
         <v>2.098575</v>
       </c>
       <c r="F101" t="n">
-        <v>400568600172</v>
+        <v>400568690161</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -6519,11 +6519,11 @@
         <v>20</v>
       </c>
       <c r="L101" t="n">
-        <v>164</v>
+        <v>4490</v>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>WM PUERTA PARADA</t>
+          <t>PAIZ FRAIJANES</t>
         </is>
       </c>
       <c r="N101" t="n">
@@ -6541,11 +6541,11 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HB HELLES LAGER LATA</t>
+          <t>HB SESSION LATA</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>75437615</v>
+        <v>75437617</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -6559,7 +6559,7 @@
         <v>2.098575</v>
       </c>
       <c r="F102" t="n">
-        <v>400568600172</v>
+        <v>400568690161</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -6579,11 +6579,11 @@
         <v>20</v>
       </c>
       <c r="L102" t="n">
-        <v>1087</v>
+        <v>180</v>
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
+          <t>PAIZ HUEHUETENANGO</t>
         </is>
       </c>
       <c r="N102" t="n">
@@ -6639,11 +6639,11 @@
         <v>20</v>
       </c>
       <c r="L103" t="n">
-        <v>4126</v>
+        <v>22</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>PAIZ CHIQUIMULA PRADERA</t>
+          <t>PAIZ LAS AMERICAS</t>
         </is>
       </c>
       <c r="N103" t="n">
@@ -6699,11 +6699,11 @@
         <v>20</v>
       </c>
       <c r="L104" t="n">
-        <v>727</v>
+        <v>4491</v>
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>PAIZ COLONIA VISTA HERMOS</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N104" t="n">
@@ -6759,11 +6759,11 @@
         <v>20</v>
       </c>
       <c r="L105" t="n">
-        <v>4490</v>
+        <v>20</v>
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>PAIZ FRAIJANES</t>
+          <t>PAIZ MONTUFAR</t>
         </is>
       </c>
       <c r="N105" t="n">
@@ -6819,11 +6819,11 @@
         <v>20</v>
       </c>
       <c r="L106" t="n">
-        <v>180</v>
+        <v>458</v>
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>PAIZ HUEHUETENANGO</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N106" t="n">
@@ -6879,11 +6879,11 @@
         <v>20</v>
       </c>
       <c r="L107" t="n">
-        <v>22</v>
+        <v>4317</v>
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>PAIZ LAS AMERICAS</t>
+          <t>PAIZ SAN LUCAS</t>
         </is>
       </c>
       <c r="N107" t="n">
@@ -6939,11 +6939,11 @@
         <v>20</v>
       </c>
       <c r="L108" t="n">
-        <v>4491</v>
+        <v>4173</v>
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>PAIZ SANTA AMELIA</t>
         </is>
       </c>
       <c r="N108" t="n">
@@ -6999,11 +6999,11 @@
         <v>20</v>
       </c>
       <c r="L109" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>PAIZ MONTUFAR</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N109" t="n">
@@ -7059,11 +7059,11 @@
         <v>20</v>
       </c>
       <c r="L110" t="n">
-        <v>458</v>
+        <v>4370</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
+          <t>WM PROCERES</t>
         </is>
       </c>
       <c r="N110" t="n">
@@ -7119,11 +7119,11 @@
         <v>20</v>
       </c>
       <c r="L111" t="n">
-        <v>4317</v>
+        <v>164</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>PAIZ SAN LUCAS</t>
+          <t>WM PUERTA PARADA</t>
         </is>
       </c>
       <c r="N111" t="n">
@@ -7179,11 +7179,11 @@
         <v>20</v>
       </c>
       <c r="L112" t="n">
-        <v>4173</v>
+        <v>1087</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>PAIZ SANTA AMELIA</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N112" t="n">
@@ -7239,11 +7239,11 @@
         <v>20</v>
       </c>
       <c r="L113" t="n">
-        <v>34</v>
+        <v>460</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>PAIZ UTATLAN</t>
+          <t>WM XELA</t>
         </is>
       </c>
       <c r="N113" t="n">
@@ -7261,11 +7261,11 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>HB SESSION LATA</t>
+          <t>NC OLD RASPUTIN LATA</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>75437617</v>
+        <v>75437613</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -7273,13 +7273,13 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>16</v>
+        <v>43.8</v>
       </c>
       <c r="E114" t="n">
-        <v>2.098575</v>
+        <v>5.74485</v>
       </c>
       <c r="F114" t="n">
-        <v>400568690161</v>
+        <v>72734400410</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -7299,11 +7299,11 @@
         <v>20</v>
       </c>
       <c r="L114" t="n">
-        <v>4370</v>
+        <v>4491</v>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>WM PROCERES</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N114" t="n">
@@ -7321,11 +7321,11 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>HB SESSION LATA</t>
+          <t>NC OLD RASPUTIN LATA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>75437617</v>
+        <v>75437613</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -7333,13 +7333,13 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>16</v>
+        <v>43.8</v>
       </c>
       <c r="E115" t="n">
-        <v>2.098575</v>
+        <v>5.74485</v>
       </c>
       <c r="F115" t="n">
-        <v>400568690161</v>
+        <v>72734400410</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -7359,11 +7359,11 @@
         <v>20</v>
       </c>
       <c r="L115" t="n">
-        <v>164</v>
+        <v>458</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>WM PUERTA PARADA</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N115" t="n">
@@ -7381,11 +7381,11 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>HB SESSION LATA</t>
+          <t>NC OLD RASPUTIN LATA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>75437617</v>
+        <v>75437613</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -7393,13 +7393,13 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>16</v>
+        <v>43.8</v>
       </c>
       <c r="E116" t="n">
-        <v>2.098575</v>
+        <v>5.74485</v>
       </c>
       <c r="F116" t="n">
-        <v>400568690161</v>
+        <v>72734400410</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -7419,11 +7419,11 @@
         <v>20</v>
       </c>
       <c r="L116" t="n">
-        <v>1087</v>
+        <v>34</v>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N116" t="n">
@@ -7441,11 +7441,11 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>HB SESSION LATA</t>
+          <t>NC OLD RASPUTIN LATA</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>75437617</v>
+        <v>75437613</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -7453,13 +7453,13 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>16</v>
+        <v>43.8</v>
       </c>
       <c r="E117" t="n">
-        <v>2.098575</v>
+        <v>5.74485</v>
       </c>
       <c r="F117" t="n">
-        <v>400568690161</v>
+        <v>72734400410</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -7479,11 +7479,11 @@
         <v>20</v>
       </c>
       <c r="L117" t="n">
-        <v>460</v>
+        <v>1087</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>WM XELA</t>
+          <t>WM QUETZALTENANGO PERIFER</t>
         </is>
       </c>
       <c r="N117" t="n">
@@ -7539,11 +7539,11 @@
         <v>20</v>
       </c>
       <c r="L118" t="n">
-        <v>4491</v>
+        <v>460</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>PAIZ LIBERACION</t>
+          <t>WM XELA</t>
         </is>
       </c>
       <c r="N118" t="n">
@@ -7561,11 +7561,11 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NC OLD RASPUTIN LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>75437613</v>
+        <v>75437612</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -7579,7 +7579,7 @@
         <v>5.74485</v>
       </c>
       <c r="F119" t="n">
-        <v>72734400410</v>
+        <v>72734400408</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -7599,11 +7599,11 @@
         <v>20</v>
       </c>
       <c r="L119" t="n">
-        <v>458</v>
+        <v>4491</v>
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
+          <t>PAIZ LIBERACION</t>
         </is>
       </c>
       <c r="N119" t="n">
@@ -7621,11 +7621,11 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>NC OLD RASPUTIN LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>75437613</v>
+        <v>75437612</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -7639,7 +7639,7 @@
         <v>5.74485</v>
       </c>
       <c r="F120" t="n">
-        <v>72734400410</v>
+        <v>72734400408</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -7659,11 +7659,11 @@
         <v>20</v>
       </c>
       <c r="L120" t="n">
-        <v>34</v>
+        <v>458</v>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>PAIZ UTATLAN</t>
+          <t>PAIZ SALIDA AL PACIFICO</t>
         </is>
       </c>
       <c r="N120" t="n">
@@ -7681,11 +7681,11 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>NC OLD RASPUTIN LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>75437613</v>
+        <v>75437612</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -7699,7 +7699,7 @@
         <v>5.74485</v>
       </c>
       <c r="F121" t="n">
-        <v>72734400410</v>
+        <v>72734400408</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -7719,11 +7719,11 @@
         <v>20</v>
       </c>
       <c r="L121" t="n">
-        <v>1054</v>
+        <v>34</v>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>WALMART SAN CRISTóBAL</t>
+          <t>PAIZ UTATLAN</t>
         </is>
       </c>
       <c r="N121" t="n">
@@ -7741,11 +7741,11 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>NC OLD RASPUTIN LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>75437613</v>
+        <v>75437612</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -7759,7 +7759,7 @@
         <v>5.74485</v>
       </c>
       <c r="F122" t="n">
-        <v>72734400410</v>
+        <v>72734400408</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -7801,11 +7801,11 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NC OLD RASPUTIN LATA</t>
+          <t>NC SCRIMSHAW LATA</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>75437613</v>
+        <v>75437612</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -7819,7 +7819,7 @@
         <v>5.74485</v>
       </c>
       <c r="F123" t="n">
-        <v>72734400410</v>
+        <v>72734400408</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -7853,366 +7853,6 @@
         <v>3</v>
       </c>
       <c r="P123" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B124" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E124" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F124" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H124" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I124" t="n">
-        <v>20</v>
-      </c>
-      <c r="J124" t="n">
-        <v>1</v>
-      </c>
-      <c r="K124" t="n">
-        <v>20</v>
-      </c>
-      <c r="L124" t="n">
-        <v>4491</v>
-      </c>
-      <c r="M124" t="inlineStr">
-        <is>
-          <t>PAIZ LIBERACION</t>
-        </is>
-      </c>
-      <c r="N124" t="n">
-        <v>0</v>
-      </c>
-      <c r="O124" t="n">
-        <v>3</v>
-      </c>
-      <c r="P124" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B125" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E125" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F125" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H125" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I125" t="n">
-        <v>20</v>
-      </c>
-      <c r="J125" t="n">
-        <v>1</v>
-      </c>
-      <c r="K125" t="n">
-        <v>20</v>
-      </c>
-      <c r="L125" t="n">
-        <v>458</v>
-      </c>
-      <c r="M125" t="inlineStr">
-        <is>
-          <t>PAIZ SALIDA AL PACIFICO</t>
-        </is>
-      </c>
-      <c r="N125" t="n">
-        <v>0</v>
-      </c>
-      <c r="O125" t="n">
-        <v>3</v>
-      </c>
-      <c r="P125" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B126" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E126" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F126" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H126" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I126" t="n">
-        <v>20</v>
-      </c>
-      <c r="J126" t="n">
-        <v>1</v>
-      </c>
-      <c r="K126" t="n">
-        <v>20</v>
-      </c>
-      <c r="L126" t="n">
-        <v>34</v>
-      </c>
-      <c r="M126" t="inlineStr">
-        <is>
-          <t>PAIZ UTATLAN</t>
-        </is>
-      </c>
-      <c r="N126" t="n">
-        <v>0</v>
-      </c>
-      <c r="O126" t="n">
-        <v>3</v>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B127" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E127" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F127" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H127" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I127" t="n">
-        <v>20</v>
-      </c>
-      <c r="J127" t="n">
-        <v>1</v>
-      </c>
-      <c r="K127" t="n">
-        <v>20</v>
-      </c>
-      <c r="L127" t="n">
-        <v>1054</v>
-      </c>
-      <c r="M127" t="inlineStr">
-        <is>
-          <t>WALMART SAN CRISTóBAL</t>
-        </is>
-      </c>
-      <c r="N127" t="n">
-        <v>0</v>
-      </c>
-      <c r="O127" t="n">
-        <v>3</v>
-      </c>
-      <c r="P127" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B128" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E128" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F128" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H128" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I128" t="n">
-        <v>20</v>
-      </c>
-      <c r="J128" t="n">
-        <v>1</v>
-      </c>
-      <c r="K128" t="n">
-        <v>20</v>
-      </c>
-      <c r="L128" t="n">
-        <v>1087</v>
-      </c>
-      <c r="M128" t="inlineStr">
-        <is>
-          <t>WM QUETZALTENANGO PERIFER</t>
-        </is>
-      </c>
-      <c r="N128" t="n">
-        <v>0</v>
-      </c>
-      <c r="O128" t="n">
-        <v>3</v>
-      </c>
-      <c r="P128" t="inlineStr">
-        <is>
-          <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>NC SCRIMSHAW LATA</t>
-        </is>
-      </c>
-      <c r="B129" t="n">
-        <v>75437612</v>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="E129" t="n">
-        <v>5.74485</v>
-      </c>
-      <c r="F129" t="n">
-        <v>72734400408</v>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>CLAN CERVECERO SA</t>
-        </is>
-      </c>
-      <c r="H129" t="n">
-        <v>258977</v>
-      </c>
-      <c r="I129" t="n">
-        <v>20</v>
-      </c>
-      <c r="J129" t="n">
-        <v>1</v>
-      </c>
-      <c r="K129" t="n">
-        <v>20</v>
-      </c>
-      <c r="L129" t="n">
-        <v>460</v>
-      </c>
-      <c r="M129" t="inlineStr">
-        <is>
-          <t>WM XELA</t>
-        </is>
-      </c>
-      <c r="N129" t="n">
-        <v>0</v>
-      </c>
-      <c r="O129" t="n">
-        <v>3</v>
-      </c>
-      <c r="P129" t="inlineStr">
         <is>
           <t>MEDICIÓN · sin combo ítem-tienda en maestro — requiere habilitación · piso de 1 caja</t>
         </is>
@@ -8338,16 +7978,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="F10" t="n">
-        <v>3571</v>
+        <v>3251</v>
       </c>
     </row>
     <row r="11">
@@ -8360,16 +8000,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E11" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="F11" t="n">
-        <v>34477</v>
+        <v>31630</v>
       </c>
     </row>
     <row r="12">
@@ -8380,22 +8020,22 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D12" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E12" t="n">
-        <v>3340</v>
+        <v>3220</v>
       </c>
       <c r="F12" t="n">
-        <v>69436</v>
+        <v>66269</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NOTA: 11 tiendas con incidencias abiertas (ajustes de inventario, planograma, reclamos) quedan</t>
+          <t>NOTA: 12 tiendas con incidencias abiertas (ajustes de inventario, planograma, reclamos) quedan</t>
         </is>
       </c>
     </row>

</xml_diff>